<commit_message>
Remove unit price from Yellowstone client budget
Client sheet and PDF now show only the package total (USD 61,500),
with structure included and no per-account price.

Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-yellowstone-cliente.xlsx
+++ b/docs/presupuesto-yellowstone-cliente.xlsx
@@ -10,7 +10,7 @@
     <sheet name="PRESUPUESTO" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRESUPUESTO'!$A$1:$G$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRESUPUESTO'!$A$1:$E$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -112,12 +112,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2E8F0"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -190,42 +190,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -240,11 +239,9 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -614,19 +611,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E38"/>
+  <dimension ref="B2:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="2.2" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="2" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="8" customHeight="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -673,7 +667,7 @@
       </c>
       <c r="E7" s="6" t="n"/>
     </row>
-    <row r="8" ht="18" customHeight="1">
+    <row r="8">
       <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Modalidad</t>
@@ -691,7 +685,7 @@
       </c>
       <c r="E8" s="9" t="n"/>
     </row>
-    <row r="9" ht="18" customHeight="1">
+    <row r="9">
       <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Cuentas orgánicas</t>
@@ -709,7 +703,7 @@
       </c>
       <c r="E9" s="9" t="n"/>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10">
       <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Moneda</t>
@@ -735,29 +729,29 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Total (USD)</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="10" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Bots originales (cuentas orgánicas)</t>
         </is>
@@ -768,9 +762,9 @@
       <c r="D14" s="12" t="n">
         <v>61500</v>
       </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>Precio final del paquete · $20.50 c/u</t>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Precio final del paquete</t>
         </is>
       </c>
     </row>
@@ -795,29 +789,29 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Total (USD)</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="B19" s="10" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Espartanos (operación elite)</t>
         </is>
@@ -830,14 +824,14 @@
           <t>INCLUIDO</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>Capa operativa elite del proyecto</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="B20" s="10" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Red Humana</t>
         </is>
@@ -850,14 +844,14 @@
           <t>INCLUIDO</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>Red operativa permanente</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="B21" s="10" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Laboratorio Bots</t>
         </is>
@@ -870,14 +864,14 @@
           <t>INCLUIDO</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>Celda técnica y soporte de bots</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="B22" s="10" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Staff</t>
         </is>
@@ -890,14 +884,14 @@
           <t>INCLUIDO</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>Operación diaria</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="10" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Equipo Gerencia</t>
         </is>
@@ -910,7 +904,7 @@
           <t>INCLUIDO</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Dirección y control del proyecto</t>
         </is>
@@ -945,34 +939,34 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Rubro</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Total (USD)</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>Componente</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>Detalle</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>Paquete comercial (3,000 cuentas)</t>
         </is>
       </c>
-      <c r="C28" s="18">
+      <c r="C28" s="19">
         <f>D15</f>
         <v/>
       </c>
@@ -981,19 +975,19 @@
           <t>3,000</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>Cuentas orgánicas (bots originales)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Estructura operativa incluida</t>
         </is>
       </c>
-      <c r="C29" s="18" t="n">
+      <c r="C29" s="19" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -1001,19 +995,19 @@
           <t>500</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>Espartanos</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="19" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="C30" s="20">
+      <c r="C30" s="21">
         <f>C28+C29</f>
         <v/>
       </c>
@@ -1022,19 +1016,19 @@
           <t>9,000</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>Red Humana</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="21" t="inlineStr">
+      <c r="B31" s="22" t="inlineStr">
         <is>
           <t>TOTAL PRESUPUESTO</t>
         </is>
       </c>
-      <c r="C31" s="22">
+      <c r="C31" s="23">
         <f>C30</f>
         <v/>
       </c>
@@ -1043,19 +1037,19 @@
           <t>20 + 12 + 3</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>Lab Bots · Staff · Gerencia</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="23" t="inlineStr">
+      <c r="B32" s="24" t="inlineStr">
         <is>
           <t>Presupuesto all-in</t>
         </is>
       </c>
-      <c r="C32" s="24">
+      <c r="C32" s="25">
         <f>"USD "&amp;TEXT(C31,"#,##0")</f>
         <v/>
       </c>
@@ -1064,53 +1058,35 @@
           <t>All-in</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>Estructura completa incluida</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>Precio por cuenta</t>
-        </is>
-      </c>
-      <c r="C34" s="25">
-        <f>IF(C14=0,0,D14/C14)</f>
-        <v/>
-      </c>
-      <c r="D34" s="26" t="inlineStr">
+      <c r="B34" s="26" t="inlineStr">
         <is>
           <t>Precio final del paquete Yellowstone: USD 61,500 por 3,000 cuentas orgánicas, con estructura operativa completa incluida (Espartanos, Red Humana, Laboratorio Bots, Staff y Equipo de Gerencia).</t>
         </is>
       </c>
+      <c r="C34" s="14" t="n"/>
+      <c r="D34" s="14" t="n"/>
       <c r="E34" s="14" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>Cuentas incluidas</t>
-        </is>
-      </c>
-      <c r="C35" s="27">
-        <f>C14</f>
-        <v/>
-      </c>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
       <c r="D35" s="14" t="n"/>
       <c r="E35" s="14" t="n"/>
     </row>
-    <row r="36">
-      <c r="D36" s="14" t="n"/>
-      <c r="E36" s="14" t="n"/>
-    </row>
-    <row r="38">
-      <c r="B38" s="28" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="27" t="inlineStr">
         <is>
           <t>Presupuesto referencial expresado en dólares estadounidenses.</t>
         </is>
       </c>
-      <c r="D38" s="29" t="inlineStr">
+      <c r="D37" s="28" t="inlineStr">
         <is>
           <t>VIGENCIA: 15 DÍAS  |  1 / 1</t>
         </is>
@@ -1119,17 +1095,17 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D34:E36"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="B34:E35"/>
+    <mergeCell ref="D37:E37"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="D9:E9"/>
   </mergeCells>
-  <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+  <pageMargins left="0.45" right="0.45" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix WhatsApp Yellowstone budget PDF with visible total
Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-yellowstone-cliente.xlsx
+++ b/docs/presupuesto-yellowstone-cliente.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="PRESUPUESTO" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRESUPUESTO'!$A$1:$E$32</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,17 +46,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00151A22"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00151A22"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
@@ -78,7 +65,7 @@
     <font>
       <name val="Arial"/>
       <color rgb="0094A3B8"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -90,7 +77,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00C41E3A"/>
-      <sz val="18"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -111,7 +98,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -120,12 +107,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2E8F0"/>
+        <fgColor rgb="001B2A47"/>
       </patternFill>
     </fill>
     <fill>
@@ -135,7 +117,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B2A47"/>
+        <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -154,7 +136,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -176,92 +158,48 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -625,16 +563,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E26"/>
+  <dimension ref="B2:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.2" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -661,228 +598,186 @@
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Paquete: Cuentas orgánicas + estructura operativa</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Moneda</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="8" t="inlineStr">
-        <is>
           <t>CANT.</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>CONCEPTO</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E8" s="9" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="B7" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>BOTS ORIGINALES (cuentas orgánicas)</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="B8" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>ESPARTANOS (operación elite)</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="B9" s="10" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>BOTS ORIGINALES (cuentas orgánicas)</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="B9" s="5" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>RED HUMANA</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="10" t="n">
-        <v>500</v>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>ESPARTANOS (operación elite)</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="B10" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>LABORATORIO BOTS</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="5" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="10" t="n">
-        <v>9000</v>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>RED HUMANA</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="B11" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>STAFF</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>LABORATORIO BOTS</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="B12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>EQUIPO GERENCIA</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n"/>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>STAFF</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="n"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="B14" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>EQUIPO GERENCIA</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="n"/>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="B16" s="13" t="inlineStr">
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>TOTAL PRESUPUESTO</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="15" t="n">
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="10" t="n">
         <v>61500</v>
       </c>
-      <c r="E16" s="16" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="17" t="inlineStr">
+    </row>
+    <row r="16">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>RESUMEN</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Inversión total</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="14" t="n">
+        <v>61500</v>
+      </c>
     </row>
     <row r="19">
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Inversión total</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="20" t="n">
-        <v>61500</v>
-      </c>
-      <c r="E19" s="21" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="22" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="23" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>• Incluye estructura operativa: Espartanos, Red Humana, Laboratorio Bots, Staff y Equipo de Gerencia.
 • Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
 • Precio final del paquete: USD 61,500.</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="24" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="24" t="n"/>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="24" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="17" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="17" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="24" t="n"/>
-      <c r="C24" s="24" t="n"/>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="25" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>YELLOWSTONE · Presupuesto cliente · 1 hoja</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B22:E24"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D12:E12"/>
+  <mergeCells count="7">
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B20:D22"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>